<commit_message>
Updates to problems and example files.
</commit_message>
<xml_diff>
--- a/lesson06/EfficiencyGraphs.xlsx
+++ b/lesson06/EfficiencyGraphs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://webmailbyui-my.sharepoint.com/personal/ggodderi_byui_edu/Documents/Documents/CSEE/Semesters/Winter2024/CSE130/Lesson06/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://webmailbyui-my.sharepoint.com/personal/ggodderi_byui_edu/Documents/Documents/CSEE/ClassRepos/cse130Code/lesson06/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="22" documentId="8_{AADCB412-1360-4F58-9A16-EE2EC53E8541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{42F578B6-B7FA-4E62-BE48-4B72315F65B6}"/>
   <bookViews>
-    <workbookView xWindow="1560" yWindow="1560" windowWidth="25365" windowHeight="12195" xr2:uid="{DD387D85-F87D-44A9-BDBF-93CF9FA32117}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DD387D85-F87D-44A9-BDBF-93CF9FA32117}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>